<commit_message>
data: two-step simulation results for 2026-Q1 and 2026-Q2
Master CSV and latest outputs updated after two-step pipeline verification.
Step 1 Q1-only file: 2026-Q1 extracted with net assets 31/3/2026.
Step 2 Q2 file: 2026-Q2 added with net assets 30/6/2026.
Results matched manual reference at 209/210 and 280/280.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/latest/SIFA_DATA_latest.xlsx
+++ b/output/latest/SIFA_DATA_latest.xlsx
@@ -4203,36 +4203,6 @@
       <c r="U4" t="n">
         <v>80868.03999999999</v>
       </c>
-      <c r="V4" t="n">
-        <v>-3.23083364820021</v>
-      </c>
-      <c r="W4" t="n">
-        <v>31.6123166833399</v>
-      </c>
-      <c r="X4" t="n">
-        <v>-3.94380367943874</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>40.0760053044441</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>-16.6352244965996</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>26.3989582155076</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>3.18358154840899</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>12.8899718532315</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>9.649028219306389</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>100</v>
-      </c>
       <c r="AF4" t="n">
         <v>683449.042811719</v>
       </c>

</xml_diff>